<commit_message>
Stress-test answer key: add scale results for 120 to 2,000 documents
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018tZ332BrVjw95yfzUCJnvR
</commit_message>
<xml_diff>
--- a/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
+++ b/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Documents" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Key dates" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Must-find passages" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Scale results" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Documents'!$A$1:$R$121</definedName>
@@ -14285,4 +14286,357 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Upload + index (s)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Stage 02 list (s)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Readiness check, all (s)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Readiness check, attorney set (s)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Analysis (s)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Total run (s)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Browser storage (MB)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>JS heap (MB)</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Pass 1 state</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Pass 1 held</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Intruders caught (of 2)</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Chronology events</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Console errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>120</v>
+      </c>
+      <c r="B2" t="n">
+        <v>117</v>
+      </c>
+      <c r="C2" t="n">
+        <v>9.101000000000001</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.453</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="G2" t="n">
+        <v>12.725</v>
+      </c>
+      <c r="H2" t="n">
+        <v>41</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>CURE REQUIRED</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="n">
+        <v>194</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>250</v>
+      </c>
+      <c r="B3" t="n">
+        <v>247</v>
+      </c>
+      <c r="C3" t="n">
+        <v>12.191</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.5659999999999999</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.384</v>
+      </c>
+      <c r="G3" t="n">
+        <v>29.097</v>
+      </c>
+      <c r="H3" t="n">
+        <v>63</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>CURE REQUIRED</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>373</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>500</v>
+      </c>
+      <c r="B4" t="n">
+        <v>497</v>
+      </c>
+      <c r="C4" t="n">
+        <v>21.368</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.866</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.678</v>
+      </c>
+      <c r="G4" t="n">
+        <v>64.486</v>
+      </c>
+      <c r="H4" t="n">
+        <v>112</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>CURE REQUIRED</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="n">
+        <v>717</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B5" t="n">
+        <v>997</v>
+      </c>
+      <c r="C5" t="n">
+        <v>34.705</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.694</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.682</v>
+      </c>
+      <c r="G5" t="n">
+        <v>156.005</v>
+      </c>
+      <c r="H5" t="n">
+        <v>230</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J5" t="n">
+        <v>119.8</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>CURE REQUIRED</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1394</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1997</v>
+      </c>
+      <c r="C6" t="n">
+        <v>51.282</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.686</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5.138</v>
+      </c>
+      <c r="G6" t="n">
+        <v>562.212</v>
+      </c>
+      <c r="H6" t="n">
+        <v>687</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J6" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>CURE REQUIRED</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>3</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2773</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Stress-test answer key: record the post-fix run
The committed workbook showed the run from before the four fixes in #23.
It now shows the run against the fixed build: 33 PASS, 8 FINDING, 0 FAIL,
with scale results for 250 to 1,000 documents.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018tZ332BrVjw95yfzUCJnvR
</commit_message>
<xml_diff>
--- a/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
+++ b/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
@@ -54,7 +54,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -64,11 +64,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E3A5F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
     <fill>
@@ -99,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -123,9 +118,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -632,14 +624,14 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>AUTOMATED RUN: 2026-09-25 00:18 UTC, 120 files, 41 s</t>
+          <t>AUTOMATED RUN: 2026-09-25 00:43 UTC, 120 files, 43 s</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Results: 24 PASS, 4 FAIL, 8 FINDING</t>
+          <t>Results: 33 PASS, 0 FAIL, 8 FINDING</t>
         </is>
       </c>
     </row>
@@ -654,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -715,12 +707,12 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>117 entered; wrongly skipped as duplicates: 2025-02-19 Site sign-in sheet (scan).pdf; 2025-02-20 Voicemail transcript - Whitcomb.txt</t>
+          <t>119</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -750,7 +742,7 @@
           <t>Daily report 02-03-2025 (copy from superintendent laptop).txt was already ingested — skipped.</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -774,15 +766,15 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>1 notice(s)</t>
+          <t>2 notice(s)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -814,7 +806,7 @@
           <t>41 of 48 match; differs: 2024-04-01 Notice to Proceed - Harpeth Ridge.pdf -&gt; AGREEMENT; 2024-11-08 Change Order 14 - MRI Suite Redesign (signed scan).pdf -&gt; DOCUMENT; 2024-12-20 Brightwater Request for Time Extension - CO 14.pdf -&gt; AGREEMENT; 2025-01-28 RFI-087 - Substitution request 22 ga supply trunks.pdf -&gt; DOCUMENT; 2025-09-12 Certificate of Substantial Completion.pdf -&gt; AGREEMENT; 2025-10-15 Pay Application No. 18 with wire instructions.pdf -&gt; DOCUMENT; Keystone delay notice (legacy export, Windows-1252).txt -&gt; DOCUMENT</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -846,7 +838,7 @@
           <t>31 of 31</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -870,15 +862,15 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>LIKELY 106, POSSIBLE 5, OUT OF PERIOD 1, NO MATCH 5</t>
+          <t>LIKELY 106, POSSIBLE 5, OUT OF PERIOD 1, NO MATCH 7</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>LIKELY 106, POSSIBLE 5, OUT OF PERIOD 1, NO MATCH 5</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
+          <t>LIKELY 106, POSSIBLE 5, OUT OF PERIOD 1, NO MATCH 7</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -910,7 +902,7 @@
           <t>All match</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -942,7 +934,7 @@
           <t>POSSIBLE</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -974,7 +966,7 @@
           <t>OUT OF PERIOD</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1006,7 +998,7 @@
           <t>NO MATCH</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1038,7 +1030,7 @@
           <t>NO MATCH</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -1070,7 +1062,7 @@
           <t>NO MATCH</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -1102,7 +1094,7 @@
           <t>111 selected · 107 producible · 4 withheld</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1134,7 +1126,7 @@
           <t>2025-02-07 Keystone certified payroll WE 02-07-2025.csv, 2025-10-15 Pay Application No. 18 with wire instructions.pdf</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1166,7 +1158,7 @@
           <t>Produce (attorney call; the tool does not decide privilege)</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1198,7 +1190,7 @@
           <t>Produce (attorney call; the tool does not decide privilege)</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1230,7 +1222,7 @@
           <t>Scanned image with no text layer</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1259,17 +1251,17 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>not in matter</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>Scanned image with no text layer</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Never reached Stage 03: it was skipped at upload as a false duplicate (see Stage 01).</t>
+          <t>Blocking defect; the document cannot be produced as it stands.</t>
         </is>
       </c>
     </row>
@@ -1291,17 +1283,17 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>not in matter</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>No readable text</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Never reached Stage 03: it was skipped at upload as a false duplicate (see Stage 01).</t>
+          <t>Blocking defect; the document cannot be produced as it stands.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1318,7 @@
           <t>Corrupted character encoding</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1350,22 +1342,22 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Does not appear to belong to this matter</t>
+          <t>Held as not belonging to this matter (either test)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>not held</t>
+          <t>Names no party or key term of this matter</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>DEFECT FOUND: this letter comes from our own law firm (Mabry &amp; Colquitt) for another client. It shares the firm name, "LLP", "client" and "attorney" with our privileged emails, so the cohesion test sees it as related. A misfiled document from the same firm is the most likely real-world intruder. Screening (NO MATCH) is the only thing that catches it.</t>
+          <t>Blocking defect; the document cannot be produced as it stands.</t>
         </is>
       </c>
     </row>
@@ -1382,15 +1374,15 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
+          <t>Held as not belonging to this matter (either test)</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
           <t>Does not appear to belong to this matter</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Does not appear to belong to this matter</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1409,27 +1401,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Nothing else held back</t>
+          <t>Held: 2025-02-18 Text messages - Carranza to Haldane.txt</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Held as not belonging to this matter (either test)</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
+          <t>Names no party or key term of this matter</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Anything listed here was held by the cohesion test. Review whether it truly belongs to another matter.</t>
+          <t>Readable, but matches none of the screening criteria. Held until the attorney confirms it belongs; released with one click if it does.</t>
         </is>
       </c>
     </row>
@@ -1441,91 +1433,91 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Overall state</t>
+          <t>Held: 2025-05-05 Nashville construction market newsletter.eml</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>CURE REQUIRED</t>
+          <t>Held as not belonging to this matter (either test)</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>CURE REQUIRED</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
+          <t>Names no party or key term of this matter</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Under 25% unreadable, so cure rather than re-collect.</t>
+          <t>Readable, but matches none of the screening criteria. Held until the attorney confirms it belongs; released with one click if it does.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>03 Readiness (pass 2: attorney selection)</t>
+          <t>03 Readiness (pass 1: all selected)</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Held back</t>
+          <t>Nothing else held back</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Keystone delay notice (legacy export, Windows-1252).txt: Corrupted character encoding</t>
+          <t>None</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Keystone delay notice (legacy export, Windows-1252).txt: Corrupted character encoding</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Only the corrupt export should be held. The scans and intruders were already excluded by screening.</t>
+          <t>Anything listed here was held by the cohesion test. Review whether it truly belongs to another matter.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>03 Readiness (pass 2: attorney selection)</t>
+          <t>03 Readiness (pass 1: all selected)</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Advisory "No date found" lists</t>
+          <t>Overall state</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Project directory - Harpeth Ridge.json; Punch list - Level 3 (walk with Architect).md; Manufacturer data sheet - galvanized duct gauges.pdf</t>
+          <t>CURE REQUIRED</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>7 contain no recognizable date.</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
+          <t>CURE REQUIRED</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Advisory only; never blocks.</t>
+          <t>Under 25% unreadable, so cure rather than re-collect.</t>
         </is>
       </c>
     </row>
@@ -1537,119 +1529,123 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Advisory "Very short documents" lists</t>
+          <t>A NO MATCH document the attorney added by hand is held for confirmation</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>2025-02-18 Text messages - Carranza to Haldane.txt</t>
+          <t>2025-02-18 Text messages - Carranza to Haldane.txt: Names no party or key term of this matter</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>1 contain little text and may be partial exports.</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
+          <t>Names no party or key term of this matter</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Advisory only; never blocks.</t>
+          <t>The attorney confirms it belongs ("This document belongs to the matter"), which is written to the audit log, and it is released.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>04 Chronology</t>
+          <t>03 Readiness (pass 2: attorney selection)</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Dated events assembled</t>
+          <t>Held back</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>See "Key dates" sheet for the dates that matter</t>
+          <t>Keystone delay notice (legacy export, Windows-1252).txt: Corrupted character encoding</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>194</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr"/>
+          <t>Keystone delay notice (legacy export, Windows-1252).txt: Corrupted character encoding</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>After the attorney confirms the text messages, only the corrupt export should be held. The scans and intruders were already excluded by screening.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>04 Chronology</t>
+          <t>03 Readiness (pass 2: attorney selection)</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Impossible date 02/30/2025 rejected</t>
+          <t>Advisory "No date found" lists</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>1 event from the Jan 15 daily report (not 2)</t>
+          <t>Project directory - Harpeth Ridge.json; Punch list - Level 3 (walk with Architect).md; Manufacturer data sheet - galvanized duct gauges.pdf</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
+          <t>7 contain no recognizable date.</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>A rolled-over date would be a confident wrong entry.</t>
+          <t>Advisory only; never blocks.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>04 Chronology</t>
+          <t>03 Readiness (pass 2: attorney selection)</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>UK day-first date 04/03/2025 (true date March 4, 2025)</t>
+          <t>Advisory "Very short documents" lists</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>3/4/2025</t>
+          <t>2025-02-18 Text messages - Carranza to Haldane.txt</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>4/3/2025</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>1 contain little text and may be partial exports.</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>FINDING if 4/3/2025: numeric dates are always read US month-first. A foreign sender puts the event a month off.</t>
+          <t>Advisory only; never blocks.</t>
         </is>
       </c>
     </row>
@@ -1661,29 +1657,25 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Withheld documents excluded from the chronology</t>
+          <t>Dated events assembled</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>0 events from withheld documents</t>
+          <t>See "Key dates" sheet for the dates that matter</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>Privileged content must never reach analysis.</t>
-        </is>
-      </c>
+          <t>194</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -1693,219 +1685,219 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Email sent dates (RFC header format) on the chronology</t>
+          <t>Impossible date 02/30/2025 rejected</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Feb 3, 2025 and Dec 19, 2024 (a reviewer dates emails by when they were sent)</t>
+          <t>1 event from the Jan 15 daily report (not 2)</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml: 0 events, 2024-12-19 Oyelaran to Haldane - CO 14 notice window.eml: 0 events</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>FINDING: email "Date:" headers ("Mon, 3 Feb 2025") are not a format the date reader accepts, so the two hottest emails are not on the timeline at all.</t>
+          <t>A rolled-over date would be a confident wrong entry.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>05 Citations</t>
+          <t>04 Chronology</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Must-find passages surfaced by the extractor</t>
+          <t>UK day-first date 04/03/2025 (true date March 4, 2025)</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>27 passages across the hot documents</t>
+          <t>3/4/2025</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>11 found, 16 missed</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
+          <t>4/3/2025</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>See the "Must-find passages" sheet. A miss can still be added by hand in Stage 05.</t>
+          <t>FINDING if 4/3/2025: numeric dates are always read US month-first. A foreign sender puts the event a month off.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>05 Citations</t>
+          <t>04 Chronology</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Citations in multi-page PDFs point to where the passage is</t>
+          <t>Withheld documents excluded from the chronology</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>A page (or page and line) for each citation</t>
+          <t>0 events from withheld documents</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>1 of 1 multi-page PDFs cite every passage as "Line 1": 2024-03-15 Prime Contract - Tallis-Brightwater (executed).pdf</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>DEFECT FOUND: PDF text is extracted as one line per page, so every citation on page 1 reads "Line 1" and a passage on page 2 reads "Line 3". In a brief, "BWB-000001, Line 1" does not tell the reader where to look. Fix: cite PDFs by page.</t>
+          <t>Privileged content must never reach analysis.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>05 Citations</t>
+          <t>04 Chronology</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Every hot document yields at least one citation</t>
+          <t>Email sent dates (RFC header format) on the chronology</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>All hot documents cited</t>
+          <t>Feb 3, 2025 and Dec 19, 2024 (a reviewer dates emails by when they were sent)</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml; 2025-02-03 Haldane to Carranza - RE L3 supply trunks.eml</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
+          <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml: 0 events, 2024-12-19 Oyelaran to Haldane - CO 14 notice window.eml: 0 events</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>FINDING: the extractor ranks sentences by dates, dollar amounts, full names and legal verbs. Plain-language admissions ("We ran 22 gauge", "Don't hold up the ceiling grid") carry none of those, so the two most damaging emails in the case get no citation at all. The attorney must add them by hand in Stage 05.</t>
+          <t>FINDING: email "Date:" headers ("Mon, 3 Feb 2025") are not a format the date reader accepts, so the two hottest emails are not on the timeline at all.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>08 Package</t>
+          <t>05 Citations</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Privilege log lists every withheld and redacted document, with basis</t>
+          <t>Must-find passages surfaced by the extractor</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>6 entries</t>
+          <t>27 passages across the hot documents</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>6 of 6 present</t>
+          <t>11 found, 16 missed</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FINDING</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>FRCP 26(b)(5)(A).</t>
+          <t>See the "Must-find passages" sheet. A miss can still be added by hand in Stage 05.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>08 Package</t>
+          <t>05 Citations</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Other client's documents absent from the production index</t>
+          <t>Citations in multi-page PDFs point to where the passage is</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>None present</t>
+          <t>A page for each citation</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>None present</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
+          <t>All cite by page. 2024-03-15 Prime Contract - Tallis-Brightwater (executed).pdf: Page 1, Page 1, Page 1</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Confidentiality.</t>
+          <t>DEFECT FOUND: PDF text is extracted as one line per page, so every citation on page 1 reads "Line 1" and a passage on page 2 reads "Line 3". In a brief, "BWB-000001, Line 1" does not tell the reader where to look. Fix: cite PDFs by page.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>08 Package</t>
+          <t>05 Citations</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Redacted documents listed in the production index (they are produced)</t>
+          <t>Every hot document yields at least one citation</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>2025-02-07 Keystone certified payroll WE 02-07-2025.csv; 2025-10-15 Pay Application No. 18 with wire instructions.pdf</t>
+          <t>All hot documents cited</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Missing: 2025-02-07 Keystone certified payroll WE 02-07-2025.csv; 2025-10-15 Pay Application No. 18 with wire instructions.pdf</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml; 2025-02-03 Haldane to Carranza - RE L3 supply trunks.eml</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>FINDING</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>DEFECT FOUND if missing: the index includes only documents marked "produce", so a document produced in redacted form carries a Bates number but appears on neither the index nor as produced. Opposing counsel receives pages the index does not account for.</t>
+          <t>FINDING: the extractor ranks sentences by dates, dollar amounts, full names and legal verbs. Plain-language admissions ("We ran 22 gauge", "Don't hold up the ceiling grid") carry none of those, so the two most damaging emails in the case get no citation at all. The attorney must add them by hand in Stage 05.</t>
         </is>
       </c>
     </row>
@@ -1917,81 +1909,177 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Withheld documents not marked for production in the index</t>
+          <t>Privilege log lists every withheld and redacted document, with basis</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>6 entries</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
+          <t>6 of 6 present</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr"/>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>FRCP 26(b)(5)(A).</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>07 Bates</t>
+          <t>08 Package</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Bates numbers unique and prefixed BWB</t>
+          <t>Other client's documents absent from the production index</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>117 unique, all BWB-</t>
+          <t>None present</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>117 unique; prefixes ['BWB']</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
+          <t>None present</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr"/>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Confidentiality.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
+          <t>08 Package</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Redacted documents listed in the production index (they are produced)</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>2025-02-07 Keystone certified payroll WE 02-07-2025.csv; 2025-10-15 Pay Application No. 18 with wire instructions.pdf</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Both present</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>DEFECT FOUND if missing: the index includes only documents marked "produce", so a document produced in redacted form carries a Bates number but appears on neither the index nor as produced. Opposing counsel receives pages the index does not account for.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>08 Package</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Withheld documents not marked for production in the index</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>07 Bates</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Bates numbers unique and prefixed BWB</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>119 unique, all BWB-</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>119 unique; prefixes ['BWB']</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Console errors during the run</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E42" s="7" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr"/>
+      <c r="F45" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2199,7 +2287,7 @@
       <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>2024-03-15 Prime Contract - Tallis-Brightwater (executed).pdf</t>
         </is>
@@ -2347,7 +2435,7 @@
       <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>2024-04-22 Subcontract - Brightwater-Keystone HVAC.docx</t>
         </is>
@@ -2419,7 +2507,7 @@
       <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>2024-11-08 Change Order 14 - MRI Suite Redesign (draft).docx</t>
         </is>
@@ -2563,7 +2651,7 @@
       <c r="A8" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>2024-12-04 OAC Meeting Minutes No. 35.pdf</t>
         </is>
@@ -2719,7 +2807,7 @@
       <c r="A10" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>2024-12-19 Oyelaran to Haldane - CO 14 notice window.eml</t>
         </is>
@@ -2799,7 +2887,7 @@
       <c r="A11" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>2024-12-20 Brightwater Request for Time Extension - CO 14.pdf</t>
         </is>
@@ -2871,7 +2959,7 @@
       <c r="A12" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>2025-01-10 Lindqvist Rowe - extension request untimely.eml</t>
         </is>
@@ -3019,7 +3107,7 @@
       <c r="A14" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>2025-01-28 RFI-087 - Substitution request 22 ga supply trunks.pdf</t>
         </is>
@@ -3095,7 +3183,7 @@
       <c r="A15" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml</t>
         </is>
@@ -3167,7 +3255,7 @@
       <c r="A16" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>2025-02-03 Haldane to Carranza - RE L3 supply trunks.eml</t>
         </is>
@@ -3407,7 +3495,7 @@
       <c r="A19" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>2025-02-19 Meridian Cx - Duct pressure test report Level 3.pdf</t>
         </is>
@@ -3501,7 +3589,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>not in matter</t>
+          <t>DOCUMENT</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -3509,7 +3597,11 @@
           <t>NO MATCH</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>NO MATCH</t>
+        </is>
+      </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3569,7 +3661,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>not in matter</t>
+          <t>DOCUMENT</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -3577,7 +3669,11 @@
           <t>NO MATCH</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>NO MATCH</t>
+        </is>
+      </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3763,7 +3859,7 @@
       <c r="A24" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>2025-02-24 Recorded interview - Luis Carranza (QA).txt</t>
         </is>
@@ -3911,7 +4007,7 @@
       <c r="A26" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>2025-03-03 Keystone position letter - installed per submittals.docx</t>
         </is>
@@ -4059,7 +4155,7 @@
       <c r="A28" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>2025-03-11 Keystone remediation proposal - Level 3 ductwork.pdf</t>
         </is>
@@ -4683,7 +4779,7 @@
       <c r="A36" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>2025-06-30 Oyelaran - schedule status internal.eml</t>
         </is>
@@ -4755,7 +4851,7 @@
       <c r="A37" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="10" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>2025-09-12 Certificate of Substantial Completion.pdf</t>
         </is>
@@ -4827,7 +4923,7 @@
       <c r="A38" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="10" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>2025-09-26 Tallis - Notice of Liquidated Damages.pdf</t>
         </is>
@@ -5211,7 +5307,7 @@
       <c r="A43" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="10" t="inlineStr">
+      <c r="B43" s="9" t="inlineStr">
         <is>
           <t>Daily Field Report 2025-02-03 No. 213.txt</t>
         </is>
@@ -5875,7 +5971,7 @@
       <c r="A52" s="5" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="10" t="inlineStr">
+      <c r="B52" s="9" t="inlineStr">
         <is>
           <t>Submittal 005 - 23 31 13 Metal ducts.docx</t>
         </is>
@@ -10799,7 +10895,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10836,7 +10932,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10873,7 +10969,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10910,7 +11006,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10947,7 +11043,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10984,7 +11080,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11021,7 +11117,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11058,7 +11154,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11095,7 +11191,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11132,7 +11228,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11169,7 +11265,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11206,7 +11302,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11243,7 +11339,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11280,7 +11376,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11317,7 +11413,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11354,7 +11450,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11391,7 +11487,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11428,7 +11524,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11465,7 +11561,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11502,7 +11598,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11539,7 +11635,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11576,7 +11672,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11613,7 +11709,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11650,7 +11746,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11687,7 +11783,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11724,7 +11820,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11761,7 +11857,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11798,7 +11894,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11835,7 +11931,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11872,7 +11968,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11909,7 +12005,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11946,7 +12042,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11983,7 +12079,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12020,7 +12116,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G35" s="7" t="inlineStr">
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12057,7 +12153,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G36" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12094,7 +12190,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12131,7 +12227,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12168,7 +12264,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G39" s="7" t="inlineStr">
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12205,7 +12301,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G40" s="7" t="inlineStr">
+      <c r="G40" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12242,7 +12338,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12279,7 +12375,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G42" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12316,7 +12412,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G43" s="7" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12353,7 +12449,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G44" s="7" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12390,7 +12486,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="G45" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12427,7 +12523,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12464,7 +12560,7 @@
           <t>Yes (as 4/3/2025)</t>
         </is>
       </c>
-      <c r="G47" s="8" t="inlineStr">
+      <c r="G47" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -12501,7 +12597,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="G48" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12538,7 +12634,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="G49" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12575,7 +12671,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12612,7 +12708,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12649,7 +12745,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12686,7 +12782,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G53" s="7" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12723,7 +12819,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="G54" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12760,7 +12856,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G55" s="7" t="inlineStr">
+      <c r="G55" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12797,7 +12893,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12834,7 +12930,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12871,7 +12967,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="G58" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12908,7 +13004,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G59" s="7" t="inlineStr">
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12945,7 +13041,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G60" s="7" t="inlineStr">
+      <c r="G60" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12982,7 +13078,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G61" s="7" t="inlineStr">
+      <c r="G61" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13019,7 +13115,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G62" s="7" t="inlineStr">
+      <c r="G62" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13056,7 +13152,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G63" s="7" t="inlineStr">
+      <c r="G63" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13093,7 +13189,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="G64" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13130,7 +13226,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G65" s="7" t="inlineStr">
+      <c r="G65" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13167,7 +13263,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G66" s="7" t="inlineStr">
+      <c r="G66" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13204,7 +13300,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G67" s="7" t="inlineStr">
+      <c r="G67" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13241,7 +13337,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G68" s="7" t="inlineStr">
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13278,7 +13374,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G69" s="7" t="inlineStr">
+      <c r="G69" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13315,7 +13411,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G70" s="7" t="inlineStr">
+      <c r="G70" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13352,7 +13448,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G71" s="7" t="inlineStr">
+      <c r="G71" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13389,7 +13485,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G72" s="7" t="inlineStr">
+      <c r="G72" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13426,7 +13522,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G73" s="7" t="inlineStr">
+      <c r="G73" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13463,7 +13559,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G74" s="7" t="inlineStr">
+      <c r="G74" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13500,7 +13596,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G75" s="7" t="inlineStr">
+      <c r="G75" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13572,10 +13668,10 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Line 1</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
+          <t>Page 1</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13602,7 +13698,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13629,7 +13725,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13656,7 +13752,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13683,7 +13779,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13710,7 +13806,7 @@
           <t>Line 25</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13737,7 +13833,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13764,7 +13860,7 @@
           <t>Line 8</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13791,7 +13887,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13818,7 +13914,7 @@
           <t>Line 11</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13845,7 +13941,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13872,7 +13968,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13899,7 +13995,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13926,7 +14022,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13953,7 +14049,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13980,7 +14076,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14007,7 +14103,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14034,7 +14130,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14061,7 +14157,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14088,7 +14184,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14115,7 +14211,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14142,7 +14238,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14169,7 +14265,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14196,7 +14292,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14223,7 +14319,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14250,7 +14346,7 @@
           <t>Line 8</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14277,7 +14373,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14294,7 +14390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14396,31 +14492,31 @@
         <v>120</v>
       </c>
       <c r="B2" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C2" t="n">
-        <v>9.101000000000001</v>
+        <v>9.114000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.013</v>
       </c>
       <c r="E2" t="n">
-        <v>0.453</v>
+        <v>0.47</v>
       </c>
       <c r="F2" t="n">
-        <v>0.308</v>
+        <v>0.443</v>
       </c>
       <c r="G2" t="n">
-        <v>12.725</v>
+        <v>12.78</v>
       </c>
       <c r="H2" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I2" t="n">
         <v>0.1</v>
       </c>
       <c r="J2" t="n">
-        <v>17.7</v>
+        <v>37.1</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -14428,10 +14524,10 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N2" t="n">
         <v>194</v>
@@ -14445,31 +14541,31 @@
         <v>250</v>
       </c>
       <c r="B3" t="n">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C3" t="n">
-        <v>12.191</v>
+        <v>13.178</v>
       </c>
       <c r="D3" t="n">
-        <v>0.023</v>
+        <v>0.026</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.526</v>
       </c>
       <c r="F3" t="n">
-        <v>0.384</v>
+        <v>0.506</v>
       </c>
       <c r="G3" t="n">
-        <v>29.097</v>
+        <v>29.734</v>
       </c>
       <c r="H3" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I3" t="n">
         <v>0.1</v>
       </c>
       <c r="J3" t="n">
-        <v>26.5</v>
+        <v>47</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -14477,10 +14573,10 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N3" t="n">
         <v>373</v>
@@ -14494,31 +14590,31 @@
         <v>500</v>
       </c>
       <c r="B4" t="n">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="C4" t="n">
-        <v>21.368</v>
+        <v>20.304</v>
       </c>
       <c r="D4" t="n">
-        <v>0.047</v>
+        <v>0.058</v>
       </c>
       <c r="E4" t="n">
-        <v>0.866</v>
+        <v>0.6870000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>0.678</v>
+        <v>0.792</v>
       </c>
       <c r="G4" t="n">
-        <v>64.486</v>
+        <v>65.89400000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="I4" t="n">
         <v>0.2</v>
       </c>
       <c r="J4" t="n">
-        <v>52.7</v>
+        <v>60.1</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -14526,10 +14622,10 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N4" t="n">
         <v>717</v>
@@ -14543,31 +14639,31 @@
         <v>1000</v>
       </c>
       <c r="B5" t="n">
-        <v>997</v>
+        <v>999</v>
       </c>
       <c r="C5" t="n">
-        <v>34.705</v>
+        <v>33.977</v>
       </c>
       <c r="D5" t="n">
-        <v>0.11</v>
+        <v>0.091</v>
       </c>
       <c r="E5" t="n">
-        <v>1.694</v>
+        <v>1.715</v>
       </c>
       <c r="F5" t="n">
-        <v>1.682</v>
+        <v>1.564</v>
       </c>
       <c r="G5" t="n">
-        <v>156.005</v>
+        <v>156.638</v>
       </c>
       <c r="H5" t="n">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="I5" t="n">
         <v>0.3</v>
       </c>
       <c r="J5" t="n">
-        <v>119.8</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -14575,64 +14671,15 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N5" t="n">
         <v>1394</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2000</v>
-      </c>
-      <c r="B6" t="n">
-        <v>1997</v>
-      </c>
-      <c r="C6" t="n">
-        <v>51.282</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="E6" t="n">
-        <v>4.686</v>
-      </c>
-      <c r="F6" t="n">
-        <v>5.138</v>
-      </c>
-      <c r="G6" t="n">
-        <v>562.212</v>
-      </c>
-      <c r="H6" t="n">
-        <v>687</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="J6" t="n">
-        <v>106.6</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>CURE REQUIRED</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" t="n">
-        <v>2773</v>
-      </c>
-      <c r="O6" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Stress-test answer key: record the post-fix run (#24)
The committed workbook showed the run from before the four fixes in #23.
It now shows the run against the fixed build: 33 PASS, 8 FINDING, 0 FAIL,
with scale results for 250 to 1,000 documents.


Claude-Session: https://claude.ai/code/session_018tZ332BrVjw95yfzUCJnvR

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
+++ b/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
@@ -54,7 +54,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -64,11 +64,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E3A5F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
     <fill>
@@ -99,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -123,9 +118,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -632,14 +624,14 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>AUTOMATED RUN: 2026-09-25 00:18 UTC, 120 files, 41 s</t>
+          <t>AUTOMATED RUN: 2026-09-25 00:43 UTC, 120 files, 43 s</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Results: 24 PASS, 4 FAIL, 8 FINDING</t>
+          <t>Results: 33 PASS, 0 FAIL, 8 FINDING</t>
         </is>
       </c>
     </row>
@@ -654,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -715,12 +707,12 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>117 entered; wrongly skipped as duplicates: 2025-02-19 Site sign-in sheet (scan).pdf; 2025-02-20 Voicemail transcript - Whitcomb.txt</t>
+          <t>119</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -750,7 +742,7 @@
           <t>Daily report 02-03-2025 (copy from superintendent laptop).txt was already ingested — skipped.</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -774,15 +766,15 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>1 notice(s)</t>
+          <t>2 notice(s)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -814,7 +806,7 @@
           <t>41 of 48 match; differs: 2024-04-01 Notice to Proceed - Harpeth Ridge.pdf -&gt; AGREEMENT; 2024-11-08 Change Order 14 - MRI Suite Redesign (signed scan).pdf -&gt; DOCUMENT; 2024-12-20 Brightwater Request for Time Extension - CO 14.pdf -&gt; AGREEMENT; 2025-01-28 RFI-087 - Substitution request 22 ga supply trunks.pdf -&gt; DOCUMENT; 2025-09-12 Certificate of Substantial Completion.pdf -&gt; AGREEMENT; 2025-10-15 Pay Application No. 18 with wire instructions.pdf -&gt; DOCUMENT; Keystone delay notice (legacy export, Windows-1252).txt -&gt; DOCUMENT</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -846,7 +838,7 @@
           <t>31 of 31</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -870,15 +862,15 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>LIKELY 106, POSSIBLE 5, OUT OF PERIOD 1, NO MATCH 5</t>
+          <t>LIKELY 106, POSSIBLE 5, OUT OF PERIOD 1, NO MATCH 7</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>LIKELY 106, POSSIBLE 5, OUT OF PERIOD 1, NO MATCH 5</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
+          <t>LIKELY 106, POSSIBLE 5, OUT OF PERIOD 1, NO MATCH 7</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -910,7 +902,7 @@
           <t>All match</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -942,7 +934,7 @@
           <t>POSSIBLE</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -974,7 +966,7 @@
           <t>OUT OF PERIOD</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1006,7 +998,7 @@
           <t>NO MATCH</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1038,7 +1030,7 @@
           <t>NO MATCH</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -1070,7 +1062,7 @@
           <t>NO MATCH</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -1102,7 +1094,7 @@
           <t>111 selected · 107 producible · 4 withheld</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1134,7 +1126,7 @@
           <t>2025-02-07 Keystone certified payroll WE 02-07-2025.csv, 2025-10-15 Pay Application No. 18 with wire instructions.pdf</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1166,7 +1158,7 @@
           <t>Produce (attorney call; the tool does not decide privilege)</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1198,7 +1190,7 @@
           <t>Produce (attorney call; the tool does not decide privilege)</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
@@ -1230,7 +1222,7 @@
           <t>Scanned image with no text layer</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1259,17 +1251,17 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>not in matter</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>Scanned image with no text layer</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Never reached Stage 03: it was skipped at upload as a false duplicate (see Stage 01).</t>
+          <t>Blocking defect; the document cannot be produced as it stands.</t>
         </is>
       </c>
     </row>
@@ -1291,17 +1283,17 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>not in matter</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>No readable text</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Never reached Stage 03: it was skipped at upload as a false duplicate (see Stage 01).</t>
+          <t>Blocking defect; the document cannot be produced as it stands.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1318,7 @@
           <t>Corrupted character encoding</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1350,22 +1342,22 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Does not appear to belong to this matter</t>
+          <t>Held as not belonging to this matter (either test)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>not held</t>
+          <t>Names no party or key term of this matter</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>DEFECT FOUND: this letter comes from our own law firm (Mabry &amp; Colquitt) for another client. It shares the firm name, "LLP", "client" and "attorney" with our privileged emails, so the cohesion test sees it as related. A misfiled document from the same firm is the most likely real-world intruder. Screening (NO MATCH) is the only thing that catches it.</t>
+          <t>Blocking defect; the document cannot be produced as it stands.</t>
         </is>
       </c>
     </row>
@@ -1382,15 +1374,15 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
+          <t>Held as not belonging to this matter (either test)</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
           <t>Does not appear to belong to this matter</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Does not appear to belong to this matter</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1409,27 +1401,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Nothing else held back</t>
+          <t>Held: 2025-02-18 Text messages - Carranza to Haldane.txt</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Held as not belonging to this matter (either test)</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
+          <t>Names no party or key term of this matter</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Anything listed here was held by the cohesion test. Review whether it truly belongs to another matter.</t>
+          <t>Readable, but matches none of the screening criteria. Held until the attorney confirms it belongs; released with one click if it does.</t>
         </is>
       </c>
     </row>
@@ -1441,91 +1433,91 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Overall state</t>
+          <t>Held: 2025-05-05 Nashville construction market newsletter.eml</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>CURE REQUIRED</t>
+          <t>Held as not belonging to this matter (either test)</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>CURE REQUIRED</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
+          <t>Names no party or key term of this matter</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Under 25% unreadable, so cure rather than re-collect.</t>
+          <t>Readable, but matches none of the screening criteria. Held until the attorney confirms it belongs; released with one click if it does.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>03 Readiness (pass 2: attorney selection)</t>
+          <t>03 Readiness (pass 1: all selected)</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Held back</t>
+          <t>Nothing else held back</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Keystone delay notice (legacy export, Windows-1252).txt: Corrupted character encoding</t>
+          <t>None</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Keystone delay notice (legacy export, Windows-1252).txt: Corrupted character encoding</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Only the corrupt export should be held. The scans and intruders were already excluded by screening.</t>
+          <t>Anything listed here was held by the cohesion test. Review whether it truly belongs to another matter.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>03 Readiness (pass 2: attorney selection)</t>
+          <t>03 Readiness (pass 1: all selected)</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Advisory "No date found" lists</t>
+          <t>Overall state</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Project directory - Harpeth Ridge.json; Punch list - Level 3 (walk with Architect).md; Manufacturer data sheet - galvanized duct gauges.pdf</t>
+          <t>CURE REQUIRED</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>7 contain no recognizable date.</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
+          <t>CURE REQUIRED</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Advisory only; never blocks.</t>
+          <t>Under 25% unreadable, so cure rather than re-collect.</t>
         </is>
       </c>
     </row>
@@ -1537,119 +1529,123 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Advisory "Very short documents" lists</t>
+          <t>A NO MATCH document the attorney added by hand is held for confirmation</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>2025-02-18 Text messages - Carranza to Haldane.txt</t>
+          <t>2025-02-18 Text messages - Carranza to Haldane.txt: Names no party or key term of this matter</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>1 contain little text and may be partial exports.</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
+          <t>Names no party or key term of this matter</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Advisory only; never blocks.</t>
+          <t>The attorney confirms it belongs ("This document belongs to the matter"), which is written to the audit log, and it is released.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>04 Chronology</t>
+          <t>03 Readiness (pass 2: attorney selection)</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Dated events assembled</t>
+          <t>Held back</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>See "Key dates" sheet for the dates that matter</t>
+          <t>Keystone delay notice (legacy export, Windows-1252).txt: Corrupted character encoding</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>194</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr"/>
+          <t>Keystone delay notice (legacy export, Windows-1252).txt: Corrupted character encoding</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>After the attorney confirms the text messages, only the corrupt export should be held. The scans and intruders were already excluded by screening.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>04 Chronology</t>
+          <t>03 Readiness (pass 2: attorney selection)</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Impossible date 02/30/2025 rejected</t>
+          <t>Advisory "No date found" lists</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>1 event from the Jan 15 daily report (not 2)</t>
+          <t>Project directory - Harpeth Ridge.json; Punch list - Level 3 (walk with Architect).md; Manufacturer data sheet - galvanized duct gauges.pdf</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
+          <t>7 contain no recognizable date.</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>A rolled-over date would be a confident wrong entry.</t>
+          <t>Advisory only; never blocks.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>04 Chronology</t>
+          <t>03 Readiness (pass 2: attorney selection)</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>UK day-first date 04/03/2025 (true date March 4, 2025)</t>
+          <t>Advisory "Very short documents" lists</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>3/4/2025</t>
+          <t>2025-02-18 Text messages - Carranza to Haldane.txt</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>4/3/2025</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>1 contain little text and may be partial exports.</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>FINDING if 4/3/2025: numeric dates are always read US month-first. A foreign sender puts the event a month off.</t>
+          <t>Advisory only; never blocks.</t>
         </is>
       </c>
     </row>
@@ -1661,29 +1657,25 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Withheld documents excluded from the chronology</t>
+          <t>Dated events assembled</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>0 events from withheld documents</t>
+          <t>See "Key dates" sheet for the dates that matter</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>Privileged content must never reach analysis.</t>
-        </is>
-      </c>
+          <t>194</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -1693,219 +1685,219 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Email sent dates (RFC header format) on the chronology</t>
+          <t>Impossible date 02/30/2025 rejected</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Feb 3, 2025 and Dec 19, 2024 (a reviewer dates emails by when they were sent)</t>
+          <t>1 event from the Jan 15 daily report (not 2)</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml: 0 events, 2024-12-19 Oyelaran to Haldane - CO 14 notice window.eml: 0 events</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>FINDING: email "Date:" headers ("Mon, 3 Feb 2025") are not a format the date reader accepts, so the two hottest emails are not on the timeline at all.</t>
+          <t>A rolled-over date would be a confident wrong entry.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>05 Citations</t>
+          <t>04 Chronology</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Must-find passages surfaced by the extractor</t>
+          <t>UK day-first date 04/03/2025 (true date March 4, 2025)</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>27 passages across the hot documents</t>
+          <t>3/4/2025</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>11 found, 16 missed</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
+          <t>4/3/2025</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>See the "Must-find passages" sheet. A miss can still be added by hand in Stage 05.</t>
+          <t>FINDING if 4/3/2025: numeric dates are always read US month-first. A foreign sender puts the event a month off.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>05 Citations</t>
+          <t>04 Chronology</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Citations in multi-page PDFs point to where the passage is</t>
+          <t>Withheld documents excluded from the chronology</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>A page (or page and line) for each citation</t>
+          <t>0 events from withheld documents</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>1 of 1 multi-page PDFs cite every passage as "Line 1": 2024-03-15 Prime Contract - Tallis-Brightwater (executed).pdf</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>DEFECT FOUND: PDF text is extracted as one line per page, so every citation on page 1 reads "Line 1" and a passage on page 2 reads "Line 3". In a brief, "BWB-000001, Line 1" does not tell the reader where to look. Fix: cite PDFs by page.</t>
+          <t>Privileged content must never reach analysis.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>05 Citations</t>
+          <t>04 Chronology</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Every hot document yields at least one citation</t>
+          <t>Email sent dates (RFC header format) on the chronology</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>All hot documents cited</t>
+          <t>Feb 3, 2025 and Dec 19, 2024 (a reviewer dates emails by when they were sent)</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml; 2025-02-03 Haldane to Carranza - RE L3 supply trunks.eml</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
+          <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml: 0 events, 2024-12-19 Oyelaran to Haldane - CO 14 notice window.eml: 0 events</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>FINDING: the extractor ranks sentences by dates, dollar amounts, full names and legal verbs. Plain-language admissions ("We ran 22 gauge", "Don't hold up the ceiling grid") carry none of those, so the two most damaging emails in the case get no citation at all. The attorney must add them by hand in Stage 05.</t>
+          <t>FINDING: email "Date:" headers ("Mon, 3 Feb 2025") are not a format the date reader accepts, so the two hottest emails are not on the timeline at all.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>08 Package</t>
+          <t>05 Citations</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Privilege log lists every withheld and redacted document, with basis</t>
+          <t>Must-find passages surfaced by the extractor</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>6 entries</t>
+          <t>27 passages across the hot documents</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>6 of 6 present</t>
+          <t>11 found, 16 missed</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FINDING</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>FRCP 26(b)(5)(A).</t>
+          <t>See the "Must-find passages" sheet. A miss can still be added by hand in Stage 05.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>08 Package</t>
+          <t>05 Citations</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Other client's documents absent from the production index</t>
+          <t>Citations in multi-page PDFs point to where the passage is</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>None present</t>
+          <t>A page for each citation</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>None present</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
+          <t>All cite by page. 2024-03-15 Prime Contract - Tallis-Brightwater (executed).pdf: Page 1, Page 1, Page 1</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Confidentiality.</t>
+          <t>DEFECT FOUND: PDF text is extracted as one line per page, so every citation on page 1 reads "Line 1" and a passage on page 2 reads "Line 3". In a brief, "BWB-000001, Line 1" does not tell the reader where to look. Fix: cite PDFs by page.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>08 Package</t>
+          <t>05 Citations</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Redacted documents listed in the production index (they are produced)</t>
+          <t>Every hot document yields at least one citation</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>2025-02-07 Keystone certified payroll WE 02-07-2025.csv; 2025-10-15 Pay Application No. 18 with wire instructions.pdf</t>
+          <t>All hot documents cited</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Missing: 2025-02-07 Keystone certified payroll WE 02-07-2025.csv; 2025-10-15 Pay Application No. 18 with wire instructions.pdf</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+          <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml; 2025-02-03 Haldane to Carranza - RE L3 supply trunks.eml</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>FINDING</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>DEFECT FOUND if missing: the index includes only documents marked "produce", so a document produced in redacted form carries a Bates number but appears on neither the index nor as produced. Opposing counsel receives pages the index does not account for.</t>
+          <t>FINDING: the extractor ranks sentences by dates, dollar amounts, full names and legal verbs. Plain-language admissions ("We ran 22 gauge", "Don't hold up the ceiling grid") carry none of those, so the two most damaging emails in the case get no citation at all. The attorney must add them by hand in Stage 05.</t>
         </is>
       </c>
     </row>
@@ -1917,81 +1909,177 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Withheld documents not marked for production in the index</t>
+          <t>Privilege log lists every withheld and redacted document, with basis</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>6 entries</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
+          <t>6 of 6 present</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr"/>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>FRCP 26(b)(5)(A).</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>07 Bates</t>
+          <t>08 Package</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Bates numbers unique and prefixed BWB</t>
+          <t>Other client's documents absent from the production index</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>117 unique, all BWB-</t>
+          <t>None present</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>117 unique; prefixes ['BWB']</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="inlineStr">
+          <t>None present</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr"/>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Confidentiality.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
+          <t>08 Package</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Redacted documents listed in the production index (they are produced)</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>2025-02-07 Keystone certified payroll WE 02-07-2025.csv; 2025-10-15 Pay Application No. 18 with wire instructions.pdf</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Both present</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>DEFECT FOUND if missing: the index includes only documents marked "produce", so a document produced in redacted form carries a Bates number but appears on neither the index nor as produced. Opposing counsel receives pages the index does not account for.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>08 Package</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Withheld documents not marked for production in the index</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>07 Bates</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Bates numbers unique and prefixed BWB</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>119 unique, all BWB-</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>119 unique; prefixes ['BWB']</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Console errors during the run</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E42" s="7" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr"/>
+      <c r="F45" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2199,7 +2287,7 @@
       <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>2024-03-15 Prime Contract - Tallis-Brightwater (executed).pdf</t>
         </is>
@@ -2347,7 +2435,7 @@
       <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>2024-04-22 Subcontract - Brightwater-Keystone HVAC.docx</t>
         </is>
@@ -2419,7 +2507,7 @@
       <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>2024-11-08 Change Order 14 - MRI Suite Redesign (draft).docx</t>
         </is>
@@ -2563,7 +2651,7 @@
       <c r="A8" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>2024-12-04 OAC Meeting Minutes No. 35.pdf</t>
         </is>
@@ -2719,7 +2807,7 @@
       <c r="A10" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>2024-12-19 Oyelaran to Haldane - CO 14 notice window.eml</t>
         </is>
@@ -2799,7 +2887,7 @@
       <c r="A11" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>2024-12-20 Brightwater Request for Time Extension - CO 14.pdf</t>
         </is>
@@ -2871,7 +2959,7 @@
       <c r="A12" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>2025-01-10 Lindqvist Rowe - extension request untimely.eml</t>
         </is>
@@ -3019,7 +3107,7 @@
       <c r="A14" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>2025-01-28 RFI-087 - Substitution request 22 ga supply trunks.pdf</t>
         </is>
@@ -3095,7 +3183,7 @@
       <c r="A15" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml</t>
         </is>
@@ -3167,7 +3255,7 @@
       <c r="A16" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>2025-02-03 Haldane to Carranza - RE L3 supply trunks.eml</t>
         </is>
@@ -3407,7 +3495,7 @@
       <c r="A19" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>2025-02-19 Meridian Cx - Duct pressure test report Level 3.pdf</t>
         </is>
@@ -3501,7 +3589,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>not in matter</t>
+          <t>DOCUMENT</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -3509,7 +3597,11 @@
           <t>NO MATCH</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>NO MATCH</t>
+        </is>
+      </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3569,7 +3661,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>not in matter</t>
+          <t>DOCUMENT</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -3577,7 +3669,11 @@
           <t>NO MATCH</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>NO MATCH</t>
+        </is>
+      </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -3763,7 +3859,7 @@
       <c r="A24" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>2025-02-24 Recorded interview - Luis Carranza (QA).txt</t>
         </is>
@@ -3911,7 +4007,7 @@
       <c r="A26" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>2025-03-03 Keystone position letter - installed per submittals.docx</t>
         </is>
@@ -4059,7 +4155,7 @@
       <c r="A28" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>2025-03-11 Keystone remediation proposal - Level 3 ductwork.pdf</t>
         </is>
@@ -4683,7 +4779,7 @@
       <c r="A36" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>2025-06-30 Oyelaran - schedule status internal.eml</t>
         </is>
@@ -4755,7 +4851,7 @@
       <c r="A37" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="10" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>2025-09-12 Certificate of Substantial Completion.pdf</t>
         </is>
@@ -4827,7 +4923,7 @@
       <c r="A38" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="10" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>2025-09-26 Tallis - Notice of Liquidated Damages.pdf</t>
         </is>
@@ -5211,7 +5307,7 @@
       <c r="A43" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="10" t="inlineStr">
+      <c r="B43" s="9" t="inlineStr">
         <is>
           <t>Daily Field Report 2025-02-03 No. 213.txt</t>
         </is>
@@ -5875,7 +5971,7 @@
       <c r="A52" s="5" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="10" t="inlineStr">
+      <c r="B52" s="9" t="inlineStr">
         <is>
           <t>Submittal 005 - 23 31 13 Metal ducts.docx</t>
         </is>
@@ -10799,7 +10895,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10836,7 +10932,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10873,7 +10969,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10910,7 +11006,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10947,7 +11043,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -10984,7 +11080,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11021,7 +11117,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11058,7 +11154,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11095,7 +11191,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11132,7 +11228,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11169,7 +11265,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11206,7 +11302,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11243,7 +11339,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11280,7 +11376,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11317,7 +11413,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11354,7 +11450,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11391,7 +11487,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11428,7 +11524,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11465,7 +11561,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11502,7 +11598,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11539,7 +11635,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11576,7 +11672,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11613,7 +11709,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11650,7 +11746,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11687,7 +11783,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11724,7 +11820,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11761,7 +11857,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11798,7 +11894,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11835,7 +11931,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11872,7 +11968,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11909,7 +12005,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11946,7 +12042,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -11983,7 +12079,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12020,7 +12116,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G35" s="7" t="inlineStr">
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12057,7 +12153,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G36" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12094,7 +12190,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12131,7 +12227,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12168,7 +12264,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G39" s="7" t="inlineStr">
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12205,7 +12301,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G40" s="7" t="inlineStr">
+      <c r="G40" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12242,7 +12338,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12279,7 +12375,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G42" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12316,7 +12412,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G43" s="7" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12353,7 +12449,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G44" s="7" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12390,7 +12486,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="G45" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12427,7 +12523,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12464,7 +12560,7 @@
           <t>Yes (as 4/3/2025)</t>
         </is>
       </c>
-      <c r="G47" s="8" t="inlineStr">
+      <c r="G47" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -12501,7 +12597,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="G48" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12538,7 +12634,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="G49" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12575,7 +12671,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12612,7 +12708,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12649,7 +12745,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12686,7 +12782,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G53" s="7" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12723,7 +12819,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="G54" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12760,7 +12856,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G55" s="7" t="inlineStr">
+      <c r="G55" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12797,7 +12893,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12834,7 +12930,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12871,7 +12967,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="G58" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12908,7 +13004,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G59" s="7" t="inlineStr">
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12945,7 +13041,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G60" s="7" t="inlineStr">
+      <c r="G60" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -12982,7 +13078,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G61" s="7" t="inlineStr">
+      <c r="G61" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13019,7 +13115,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G62" s="7" t="inlineStr">
+      <c r="G62" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13056,7 +13152,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G63" s="7" t="inlineStr">
+      <c r="G63" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13093,7 +13189,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="G64" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13130,7 +13226,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G65" s="7" t="inlineStr">
+      <c r="G65" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13167,7 +13263,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G66" s="7" t="inlineStr">
+      <c r="G66" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13204,7 +13300,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G67" s="7" t="inlineStr">
+      <c r="G67" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13241,7 +13337,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G68" s="7" t="inlineStr">
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13278,7 +13374,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G69" s="7" t="inlineStr">
+      <c r="G69" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13315,7 +13411,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G70" s="7" t="inlineStr">
+      <c r="G70" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13352,7 +13448,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G71" s="7" t="inlineStr">
+      <c r="G71" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13389,7 +13485,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G72" s="7" t="inlineStr">
+      <c r="G72" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13426,7 +13522,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G73" s="7" t="inlineStr">
+      <c r="G73" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13463,7 +13559,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G74" s="7" t="inlineStr">
+      <c r="G74" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13500,7 +13596,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G75" s="7" t="inlineStr">
+      <c r="G75" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13572,10 +13668,10 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Line 1</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
+          <t>Page 1</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13602,7 +13698,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13629,7 +13725,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13656,7 +13752,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13683,7 +13779,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13710,7 +13806,7 @@
           <t>Line 25</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13737,7 +13833,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13764,7 +13860,7 @@
           <t>Line 8</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13791,7 +13887,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13818,7 +13914,7 @@
           <t>Line 11</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13845,7 +13941,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13872,7 +13968,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13899,7 +13995,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13926,7 +14022,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -13953,7 +14049,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -13980,7 +14076,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14007,7 +14103,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14034,7 +14130,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14061,7 +14157,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14088,7 +14184,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14115,7 +14211,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14142,7 +14238,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14169,7 +14265,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14196,7 +14292,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14223,7 +14319,7 @@
           <t>Line 1</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14250,7 +14346,7 @@
           <t>Line 8</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -14277,7 +14373,7 @@
           <t>No - add by hand in Stage 05</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>FINDING</t>
         </is>
@@ -14294,7 +14390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14396,31 +14492,31 @@
         <v>120</v>
       </c>
       <c r="B2" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C2" t="n">
-        <v>9.101000000000001</v>
+        <v>9.114000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.013</v>
       </c>
       <c r="E2" t="n">
-        <v>0.453</v>
+        <v>0.47</v>
       </c>
       <c r="F2" t="n">
-        <v>0.308</v>
+        <v>0.443</v>
       </c>
       <c r="G2" t="n">
-        <v>12.725</v>
+        <v>12.78</v>
       </c>
       <c r="H2" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I2" t="n">
         <v>0.1</v>
       </c>
       <c r="J2" t="n">
-        <v>17.7</v>
+        <v>37.1</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -14428,10 +14524,10 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N2" t="n">
         <v>194</v>
@@ -14445,31 +14541,31 @@
         <v>250</v>
       </c>
       <c r="B3" t="n">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C3" t="n">
-        <v>12.191</v>
+        <v>13.178</v>
       </c>
       <c r="D3" t="n">
-        <v>0.023</v>
+        <v>0.026</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.526</v>
       </c>
       <c r="F3" t="n">
-        <v>0.384</v>
+        <v>0.506</v>
       </c>
       <c r="G3" t="n">
-        <v>29.097</v>
+        <v>29.734</v>
       </c>
       <c r="H3" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I3" t="n">
         <v>0.1</v>
       </c>
       <c r="J3" t="n">
-        <v>26.5</v>
+        <v>47</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -14477,10 +14573,10 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N3" t="n">
         <v>373</v>
@@ -14494,31 +14590,31 @@
         <v>500</v>
       </c>
       <c r="B4" t="n">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="C4" t="n">
-        <v>21.368</v>
+        <v>20.304</v>
       </c>
       <c r="D4" t="n">
-        <v>0.047</v>
+        <v>0.058</v>
       </c>
       <c r="E4" t="n">
-        <v>0.866</v>
+        <v>0.6870000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>0.678</v>
+        <v>0.792</v>
       </c>
       <c r="G4" t="n">
-        <v>64.486</v>
+        <v>65.89400000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="I4" t="n">
         <v>0.2</v>
       </c>
       <c r="J4" t="n">
-        <v>52.7</v>
+        <v>60.1</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -14526,10 +14622,10 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N4" t="n">
         <v>717</v>
@@ -14543,31 +14639,31 @@
         <v>1000</v>
       </c>
       <c r="B5" t="n">
-        <v>997</v>
+        <v>999</v>
       </c>
       <c r="C5" t="n">
-        <v>34.705</v>
+        <v>33.977</v>
       </c>
       <c r="D5" t="n">
-        <v>0.11</v>
+        <v>0.091</v>
       </c>
       <c r="E5" t="n">
-        <v>1.694</v>
+        <v>1.715</v>
       </c>
       <c r="F5" t="n">
-        <v>1.682</v>
+        <v>1.564</v>
       </c>
       <c r="G5" t="n">
-        <v>156.005</v>
+        <v>156.638</v>
       </c>
       <c r="H5" t="n">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="I5" t="n">
         <v>0.3</v>
       </c>
       <c r="J5" t="n">
-        <v>119.8</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -14575,64 +14671,15 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N5" t="n">
         <v>1394</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2000</v>
-      </c>
-      <c r="B6" t="n">
-        <v>1997</v>
-      </c>
-      <c r="C6" t="n">
-        <v>51.282</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="E6" t="n">
-        <v>4.686</v>
-      </c>
-      <c r="F6" t="n">
-        <v>5.138</v>
-      </c>
-      <c r="G6" t="n">
-        <v>562.212</v>
-      </c>
-      <c r="H6" t="n">
-        <v>687</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="J6" t="n">
-        <v>106.6</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>CURE REQUIRED</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" t="n">
-        <v>2773</v>
-      </c>
-      <c r="O6" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Stress-test answer key: add the 2,000-document run on the fixed build
The 2,000-document tier was rerun after #23: 33 PASS, 8 FINDING, 0 FAIL,
1,999 of 2,000 files accepted (only the planted duplicate skipped), no
console errors, about 10 minutes end to end.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018tZ332BrVjw95yfzUCJnvR
</commit_message>
<xml_diff>
--- a/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
+++ b/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
@@ -14390,7 +14390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14683,6 +14683,55 @@
         <v>0</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1999</v>
+      </c>
+      <c r="C6" t="n">
+        <v>64.77500000000001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.579</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.749</v>
+      </c>
+      <c r="G6" t="n">
+        <v>451.773</v>
+      </c>
+      <c r="H6" t="n">
+        <v>595</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J6" t="n">
+        <v>165.7</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>CURE REQUIRED</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>8</v>
+      </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2773</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Stress-test answer key: add the 2,000-document run on the fixed build (#25)
The 2,000-document tier was rerun after #23: 33 PASS, 8 FINDING, 0 FAIL,
1,999 of 2,000 files accepted (only the planted duplicate skipped), no
console errors, about 10 minutes end to end.


Claude-Session: https://claude.ai/code/session_018tZ332BrVjw95yfzUCJnvR

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
+++ b/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
@@ -14390,7 +14390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14683,6 +14683,55 @@
         <v>0</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1999</v>
+      </c>
+      <c r="C6" t="n">
+        <v>64.77500000000001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.109</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.579</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.749</v>
+      </c>
+      <c r="G6" t="n">
+        <v>451.773</v>
+      </c>
+      <c r="H6" t="n">
+        <v>595</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J6" t="n">
+        <v>165.7</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>CURE REQUIRED</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>8</v>
+      </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2773</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Stress-test answer key: record the 7 Oct run on the #33 build
Re-ran the 120-document stress matter against the current build while
refreshing the product docs. The answer key now reads 35 PASS, 6 FINDING,
0 FAIL (was 33 PASS, 8 FINDING), with 228 chronology events (was 194).
The fixture documents were regenerated by generate.py; only embedded
timestamps and scan noise differ. No product code changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012TZfcNEpy1UULCR4Z9uRDv
</commit_message>
<xml_diff>
--- a/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
+++ b/testdata/stress-matter/out/120/Answer Key - 120 documents.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Stage checks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Documents" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Key dates" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Must-find passages" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Scale results" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stage checks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key dates" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Must-find passages" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scale results" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Documents'!$A$1:$R$121</definedName>
@@ -624,14 +624,14 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>AUTOMATED RUN: 2026-09-25 00:43 UTC, 120 files, 43 s</t>
+          <t>AUTOMATED RUN: 2026-10-07 18:47 UTC, 120 files, 34 s</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Results: 33 PASS, 0 FAIL, 8 FINDING</t>
+          <t>Results: 35 PASS, 0 FAIL, 6 FINDING</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>After the attorney confirms the text messages, only the corrupt export should be held. The scans and intruders were already excluded by screening.</t>
+          <t>After the attorney confirms the text messages, only the corrupt export should be held. The scans and intruders were excluded at screening and marked Not Responsive with a reason; left unmarked, each would be held as Unaccounted.</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1667,7 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>228</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>4/3/2025</t>
+          <t>2/25/2025, 4/3/2025</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>FINDING if 4/3/2025: numeric dates are always read US month-first. A foreign sender puts the event a month off.</t>
+          <t>FINDING if 4/3/2025: numeric dates are always read US month-first. A foreign sender puts the event a month off. The email's own sent date (Feb 25, 2025) is also on the chronology and is not part of this check.</t>
         </is>
       </c>
     </row>
@@ -1791,17 +1791,17 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml: 0 events, 2024-12-19 Oyelaran to Haldane - CO 14 notice window.eml: 0 events</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml: 1 events, 2024-12-19 Oyelaran to Haldane - CO 14 notice window.eml: 3 events</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>FINDING: email "Date:" headers ("Mon, 3 Feb 2025") are not a format the date reader accepts, so the two hottest emails are not on the timeline at all.</t>
+          <t>FINDING if missing: email "Date:" headers ("Mon, 3 Feb 2025") must be read so the two hottest emails are on the timeline on the day they were sent.</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>11 found, 16 missed</t>
+          <t>20 found, 7 missed</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>All cite by page. 2024-03-15 Prime Contract - Tallis-Brightwater (executed).pdf: Page 1, Page 1, Page 1</t>
+          <t>All cite by page. 2024-03-15 Prime Contract - Tallis-Brightwater (executed).pdf: Page 1, Page 1, Page 1, Page 1, Page 2, Page 2</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -1887,12 +1887,12 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>2025-02-03 Carranza to Haldane - L3 supply trunks.eml; 2025-02-03 Haldane to Carranza - RE L3 supply trunks.eml</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>All cited</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -2352,7 +2352,7 @@
       <c r="P3" s="5" t="inlineStr"/>
       <c r="Q3" s="5" t="inlineStr"/>
       <c r="R3" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="R8" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -2880,7 +2880,7 @@
         </is>
       </c>
       <c r="R10" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -3176,7 +3176,7 @@
         </is>
       </c>
       <c r="R14" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -3248,7 +3248,7 @@
         </is>
       </c>
       <c r="R15" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -3324,7 +3324,7 @@
         </is>
       </c>
       <c r="R16" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -3560,7 +3560,7 @@
       <c r="P19" s="5" t="inlineStr"/>
       <c r="Q19" s="5" t="inlineStr"/>
       <c r="R19" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -3776,7 +3776,7 @@
       <c r="P22" s="5" t="inlineStr"/>
       <c r="Q22" s="5" t="inlineStr"/>
       <c r="R22" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="Q24" s="5" t="inlineStr"/>
       <c r="R24" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -4224,7 +4224,7 @@
         </is>
       </c>
       <c r="R28" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
@@ -4300,7 +4300,7 @@
       </c>
       <c r="Q29" s="5" t="inlineStr"/>
       <c r="R29" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -4384,7 +4384,7 @@
         </is>
       </c>
       <c r="R30" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
@@ -4540,7 +4540,7 @@
       </c>
       <c r="Q32" s="5" t="inlineStr"/>
       <c r="R32" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -4844,7 +4844,7 @@
         </is>
       </c>
       <c r="R36" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
@@ -5060,7 +5060,7 @@
       <c r="P39" s="5" t="inlineStr"/>
       <c r="Q39" s="5" t="inlineStr"/>
       <c r="R39" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
@@ -5600,7 +5600,7 @@
         </is>
       </c>
       <c r="R46" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
@@ -5672,7 +5672,7 @@
         </is>
       </c>
       <c r="R47" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -5888,7 +5888,7 @@
         </is>
       </c>
       <c r="R50" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51">
@@ -6036,7 +6036,7 @@
       <c r="P52" s="5" t="inlineStr"/>
       <c r="Q52" s="5" t="inlineStr"/>
       <c r="R52" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -6308,7 +6308,7 @@
       <c r="P56" s="5" t="inlineStr"/>
       <c r="Q56" s="5" t="inlineStr"/>
       <c r="R56" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -6376,7 +6376,7 @@
       <c r="P57" s="5" t="inlineStr"/>
       <c r="Q57" s="5" t="inlineStr"/>
       <c r="R57" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58">
@@ -6580,7 +6580,7 @@
       <c r="P60" s="5" t="inlineStr"/>
       <c r="Q60" s="5" t="inlineStr"/>
       <c r="R60" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
@@ -6988,7 +6988,7 @@
       <c r="P66" s="5" t="inlineStr"/>
       <c r="Q66" s="5" t="inlineStr"/>
       <c r="R66" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="67">
@@ -7192,7 +7192,7 @@
       <c r="P69" s="5" t="inlineStr"/>
       <c r="Q69" s="5" t="inlineStr"/>
       <c r="R69" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70">
@@ -9544,7 +9544,7 @@
         </is>
       </c>
       <c r="R103" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="104">
@@ -9616,7 +9616,7 @@
         </is>
       </c>
       <c r="R104" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
@@ -9688,7 +9688,7 @@
         </is>
       </c>
       <c r="R105" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="106">
@@ -9760,7 +9760,7 @@
         </is>
       </c>
       <c r="R106" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="107">
@@ -9832,7 +9832,7 @@
         </is>
       </c>
       <c r="R107" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="108">
@@ -10584,7 +10584,7 @@
         </is>
       </c>
       <c r="R118" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="119">
@@ -10656,7 +10656,7 @@
         </is>
       </c>
       <c r="R119" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120">
@@ -10728,7 +10728,7 @@
         </is>
       </c>
       <c r="R120" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121">
@@ -10800,7 +10800,7 @@
         </is>
       </c>
       <c r="R121" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -13695,12 +13695,12 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>No - add by hand in Stage 05</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>Page 1</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -13884,7 +13884,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Page 1</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -13938,7 +13938,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Page 1</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -13965,12 +13965,12 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>No - add by hand in Stage 05</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>Line 6</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -13992,12 +13992,12 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>No - add by hand in Stage 05</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>Line 6</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -14046,7 +14046,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Page 1</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -14073,12 +14073,12 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>No - add by hand in Stage 05</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>Line 9</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -14127,12 +14127,12 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>No - add by hand in Stage 05</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>Line 25</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -14154,7 +14154,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Page 1</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -14181,12 +14181,12 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>No - add by hand in Stage 05</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>Line 9</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -14208,12 +14208,12 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>No - add by hand in Stage 05</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>Page 1</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -14235,7 +14235,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Page 1</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -14262,12 +14262,12 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>No - add by hand in Stage 05</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>Page 1</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -14289,12 +14289,12 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>No - add by hand in Stage 05</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>FINDING</t>
+          <t>Page 1</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -14316,7 +14316,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Page 1</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -14390,7 +14390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -14495,28 +14495,28 @@
         <v>119</v>
       </c>
       <c r="C2" t="n">
-        <v>9.114000000000001</v>
+        <v>10.135</v>
       </c>
       <c r="D2" t="n">
-        <v>0.013</v>
+        <v>0.015</v>
       </c>
       <c r="E2" t="n">
-        <v>0.47</v>
+        <v>0.359</v>
       </c>
       <c r="F2" t="n">
-        <v>0.443</v>
+        <v>0.464</v>
       </c>
       <c r="G2" t="n">
-        <v>12.78</v>
+        <v>0.032</v>
       </c>
       <c r="H2" t="n">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="I2" t="n">
         <v>0.1</v>
       </c>
       <c r="J2" t="n">
-        <v>37.1</v>
+        <v>46.9</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -14530,7 +14530,7 @@
         <v>2</v>
       </c>
       <c r="N2" t="n">
-        <v>194</v>
+        <v>228</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -14538,34 +14538,34 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="B3" t="n">
-        <v>249</v>
+        <v>499</v>
       </c>
       <c r="C3" t="n">
-        <v>13.178</v>
+        <v>26.378</v>
       </c>
       <c r="D3" t="n">
-        <v>0.026</v>
+        <v>0.053</v>
       </c>
       <c r="E3" t="n">
-        <v>0.526</v>
+        <v>0.778</v>
       </c>
       <c r="F3" t="n">
-        <v>0.506</v>
+        <v>0.877</v>
       </c>
       <c r="G3" t="n">
-        <v>29.734</v>
+        <v>0.149</v>
       </c>
       <c r="H3" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="J3" t="n">
-        <v>47</v>
+        <v>60.3</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -14579,7 +14579,7 @@
         <v>2</v>
       </c>
       <c r="N3" t="n">
-        <v>373</v>
+        <v>866</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -14587,34 +14587,34 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="B4" t="n">
-        <v>499</v>
+        <v>999</v>
       </c>
       <c r="C4" t="n">
-        <v>20.304</v>
+        <v>38.905</v>
       </c>
       <c r="D4" t="n">
-        <v>0.058</v>
+        <v>0.101</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6870000000000001</v>
+        <v>1.635</v>
       </c>
       <c r="F4" t="n">
-        <v>0.792</v>
+        <v>1.844</v>
       </c>
       <c r="G4" t="n">
-        <v>65.89400000000001</v>
+        <v>0.226</v>
       </c>
       <c r="H4" t="n">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="I4" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="J4" t="n">
-        <v>60.1</v>
+        <v>75.8</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -14628,7 +14628,7 @@
         <v>2</v>
       </c>
       <c r="N4" t="n">
-        <v>717</v>
+        <v>1713</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -14636,34 +14636,34 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="B5" t="n">
-        <v>999</v>
+        <v>1999</v>
       </c>
       <c r="C5" t="n">
-        <v>33.977</v>
+        <v>57.293</v>
       </c>
       <c r="D5" t="n">
-        <v>0.091</v>
+        <v>0.133</v>
       </c>
       <c r="E5" t="n">
-        <v>1.715</v>
+        <v>5.419</v>
       </c>
       <c r="F5" t="n">
-        <v>1.564</v>
+        <v>6.007</v>
       </c>
       <c r="G5" t="n">
-        <v>156.638</v>
+        <v>0.633</v>
       </c>
       <c r="H5" t="n">
-        <v>234</v>
+        <v>180</v>
       </c>
       <c r="I5" t="n">
-        <v>0.3</v>
+        <v>1.2</v>
       </c>
       <c r="J5" t="n">
-        <v>86.40000000000001</v>
+        <v>59.5</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -14677,58 +14677,9 @@
         <v>2</v>
       </c>
       <c r="N5" t="n">
-        <v>1394</v>
+        <v>3700</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2000</v>
-      </c>
-      <c r="B6" t="n">
-        <v>1999</v>
-      </c>
-      <c r="C6" t="n">
-        <v>64.77500000000001</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.109</v>
-      </c>
-      <c r="E6" t="n">
-        <v>4.579</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4.749</v>
-      </c>
-      <c r="G6" t="n">
-        <v>451.773</v>
-      </c>
-      <c r="H6" t="n">
-        <v>595</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="J6" t="n">
-        <v>165.7</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>CURE REQUIRED</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>8</v>
-      </c>
-      <c r="M6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" t="n">
-        <v>2773</v>
-      </c>
-      <c r="O6" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>